<commit_message>
Update stats for 2026-03
</commit_message>
<xml_diff>
--- a/iserv_stats.xlsx
+++ b/iserv_stats.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1066,6 +1066,32 @@
         <v>25.75459331716681</v>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="1" t="n">
+        <v>46082</v>
+      </c>
+      <c r="B28" t="n">
+        <v>6565</v>
+      </c>
+      <c r="C28" t="n">
+        <v>1022</v>
+      </c>
+      <c r="D28" t="n">
+        <v>6130599</v>
+      </c>
+      <c r="E28" t="n">
+        <v>933.8307692307692</v>
+      </c>
+      <c r="F28" t="n">
+        <v>9.782608695652172</v>
+      </c>
+      <c r="G28" t="n">
+        <v>7.805907172995785</v>
+      </c>
+      <c r="H28" t="n">
+        <v>24.5422857960095</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update stats for 2026-04
</commit_message>
<xml_diff>
--- a/iserv_stats.xlsx
+++ b/iserv_stats.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1092,6 +1092,32 @@
         <v>25.930847389865</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="1" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B29" t="n">
+        <v>6605</v>
+      </c>
+      <c r="C29" t="n">
+        <v>1027</v>
+      </c>
+      <c r="D29" t="n">
+        <v>6201476</v>
+      </c>
+      <c r="E29" t="n">
+        <v>938.9062831188494</v>
+      </c>
+      <c r="F29" t="n">
+        <v>9.535655058043124</v>
+      </c>
+      <c r="G29" t="n">
+        <v>6.314699792960665</v>
+      </c>
+      <c r="H29" t="n">
+        <v>23.4142014742895</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update stats for 2026-05
</commit_message>
<xml_diff>
--- a/iserv_stats.xlsx
+++ b/iserv_stats.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1118,6 +1118,32 @@
         <v>25.47958389063805</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="1" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B30" t="n">
+        <v>6636</v>
+      </c>
+      <c r="C30" t="n">
+        <v>1033</v>
+      </c>
+      <c r="D30" t="n">
+        <v>6305993</v>
+      </c>
+      <c r="E30" t="n">
+        <v>950.2701928872815</v>
+      </c>
+      <c r="F30" t="n">
+        <v>9.504950495049513</v>
+      </c>
+      <c r="G30" t="n">
+        <v>6.825232678386772</v>
+      </c>
+      <c r="H30" t="n">
+        <v>24.24265290867229</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update stats for 2026-06
</commit_message>
<xml_diff>
--- a/iserv_stats.xlsx
+++ b/iserv_stats.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1144,6 +1144,32 @@
         <v>25.94605585290726</v>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B31" t="n">
+        <v>6715</v>
+      </c>
+      <c r="C31" t="n">
+        <v>1039</v>
+      </c>
+      <c r="D31" t="n">
+        <v>6396549</v>
+      </c>
+      <c r="E31" t="n">
+        <v>952.57617274758</v>
+      </c>
+      <c r="F31" t="n">
+        <v>9.973796265967906</v>
+      </c>
+      <c r="G31" t="n">
+        <v>7.445708376421933</v>
+      </c>
+      <c r="H31" t="n">
+        <v>17.74227037534031</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update stats for 2026-07
</commit_message>
<xml_diff>
--- a/iserv_stats.xlsx
+++ b/iserv_stats.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1170,6 +1170,32 @@
         <v>19.97879495717576</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B32" t="n">
+        <v>6779</v>
+      </c>
+      <c r="C32" t="n">
+        <v>1054</v>
+      </c>
+      <c r="D32" t="n">
+        <v>6526524</v>
+      </c>
+      <c r="E32" t="n">
+        <v>962.7561587254758</v>
+      </c>
+      <c r="F32" t="n">
+        <v>9.356347798031939</v>
+      </c>
+      <c r="G32" t="n">
+        <v>7.551020408163267</v>
+      </c>
+      <c r="H32" t="n">
+        <v>16.93521742900779</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update stats for 2026-08
</commit_message>
<xml_diff>
--- a/iserv_stats.xlsx
+++ b/iserv_stats.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1196,6 +1196,32 @@
         <v>18.52344500830987</v>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="1" t="n">
+        <v>46235</v>
+      </c>
+      <c r="B33" t="n">
+        <v>6859</v>
+      </c>
+      <c r="C33" t="n">
+        <v>1065</v>
+      </c>
+      <c r="D33" t="n">
+        <v>6613364</v>
+      </c>
+      <c r="E33" t="n">
+        <v>964.1877824755795</v>
+      </c>
+      <c r="F33" t="n">
+        <v>9.568690095846645</v>
+      </c>
+      <c r="G33" t="n">
+        <v>7.467204843592334</v>
+      </c>
+      <c r="H33" t="n">
+        <v>16.33902488881289</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update stats for 2026-09
</commit_message>
<xml_diff>
--- a/iserv_stats.xlsx
+++ b/iserv_stats.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1222,6 +1222,32 @@
         <v>20.76541693097902</v>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B34" t="n">
+        <v>6911</v>
+      </c>
+      <c r="C34" t="n">
+        <v>1087</v>
+      </c>
+      <c r="D34" t="n">
+        <v>6882357</v>
+      </c>
+      <c r="E34" t="n">
+        <v>995.855447836782</v>
+      </c>
+      <c r="F34" t="n">
+        <v>9.646200222116462</v>
+      </c>
+      <c r="G34" t="n">
+        <v>9.027081243731194</v>
+      </c>
+      <c r="H34" t="n">
+        <v>17.31153699630203</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>